<commit_message>
Reference comparison from medianomaly.pdf T6(p.11)/T7(p.12): AUC -0.002, AP -0.001, PixAP -0.006, Dice -0.005; guide renamed REPRODUCTION_GUIDE.md
</commit_message>
<xml_diff>
--- a/artifacts/results/final_results.xlsx
+++ b/artifacts/results/final_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,17 +424,37 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Published/Reference</t>
+          <t>Paper_Term</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>Published_mean_pm_std</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>Reproduced</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Absolute_Difference</t>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Diff_rep_minus_pub</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>AbsDiff</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>PctDiff_vs_pub_mean</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Source</t>
         </is>
       </c>
     </row>
@@ -446,17 +466,37 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>N/A (no benchmark table in env)</t>
+          <t>AUC</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>0.859+-0.010</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>0.85699</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>-0.00201</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0.00201</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0.23%</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Table 6 (image-level AnoCls) p.11</t>
         </is>
       </c>
     </row>
@@ -468,17 +508,37 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>N/A (no benchmark table in env)</t>
+          <t>AP (image)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>0.934+-0.005</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>0.93286</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>-0.00114</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0.00114</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.12%</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Table 6 (image-level AnoCls) p.11</t>
         </is>
       </c>
     </row>
@@ -490,17 +550,37 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>N/A (no benchmark table in env)</t>
+          <t>pixel AUC (not reported)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>N/A (excluded by paper, p.9)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>0.96751</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>medianomaly.pdf p.9 (pixel AUC not employed)</t>
         </is>
       </c>
     </row>
@@ -512,17 +592,37 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>N/A (no benchmark table in env)</t>
+          <t>APpix</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>0.755+-0.007</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>0.74949</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>-0.00551</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0.00551</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0.73%</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Table 7 (pixel-level AnoSeg) p.12</t>
         </is>
       </c>
     </row>
@@ -534,17 +634,37 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>N/A (no benchmark table in env)</t>
+          <t>⌈Dice⌉</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>0.711+-0.006</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>0.70583</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>-0.00517</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0.00517</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.73%</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Table 7 (pixel-level AnoSeg) p.12</t>
         </is>
       </c>
     </row>
@@ -556,17 +676,37 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>N/A (no benchmark table in env)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>N/A (no published counterpart)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>0.06802</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -578,17 +718,37 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>N/A (no benchmark table in env)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>N/A (no published counterpart)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>0.00275</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -600,17 +760,37 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>N/A (no benchmark table in env)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>N/A (no published counterpart)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
           <t>0.01211</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>N/A</t>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>